<commit_message>
Zera respostas de exemplo e adiciona campo opcional Nome do Participante
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/Pesquisas_Simposio_SVP_DAP_2026.xlsx
+++ b/planilha/Pesquisas_Simposio_SVP_DAP_2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -452,13 +452,14 @@
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="28" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
     <col width="28" customWidth="1" min="26" max="26"/>
     <col width="28" customWidth="1" min="27" max="27"/>
     <col width="28" customWidth="1" min="28" max="28"/>
     <col width="28" customWidth="1" min="29" max="29"/>
     <col width="28" customWidth="1" min="30" max="30"/>
     <col width="28" customWidth="1" min="31" max="31"/>
+    <col width="28" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -474,145 +475,150 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Nome do Participante</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Posto/Graduação</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>OM/Origem</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Região Militar</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Tempo de Atuação</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Primeira Participação</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Período Realização (1-5)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Duração (1-5)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Infraestrutura Auditório (1-5)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Deslocamento HT/Evento (1-5)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Recepção e Credenciamento (1-5)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Alimentação/Coffee Break (1-5)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Conforto e Audiovisual (1-5)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Tempos Palestras (1-5)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Relevância Temas (1-5)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Qualidade Palestras (1-5)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Espaço para Dúvidas (1-5)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Clareza Normas e Sistemas (1-5)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Material de Apoio (1-5)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Avaliação Geral (1-5)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Integração Seções/DAP (1-5)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Aplicabilidade na OM (1-5)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Cumprimento Horários (1-5)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Comentários Gerais</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Pontos Fortes</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Sugestões Melhoria</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Sugestões Temas 2027</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Boas Práticas Compartilhadas</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Sugestões de Oficinas</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>

</xml_diff>